<commit_message>
Windows & Mac compatible fixes
</commit_message>
<xml_diff>
--- a/tag_manager/excel_output/html_pages_data.xlsx
+++ b/tag_manager/excel_output/html_pages_data.xlsx
@@ -456,7 +456,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>/Users/sbws_user/Documents/Webbuilder/20April/TagManger/helix_v1_v2/tag_manager/site_manager/static/site_manager/samples/www.eczee.fr/index.html</t>
+          <t>/Users/sbws_user/Documents/Custom_to_Webbuilder/helix_v1_v2/tag_manager/site_manager/static/www.eczee.fr/index.html</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -473,7 +473,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>/Users/sbws_user/Documents/Webbuilder/20April/TagManger/helix_v1_v2/tag_manager/site_manager/static/site_manager/samples/www.eczee.fr/404.html</t>
+          <t>/Users/sbws_user/Documents/Custom_to_Webbuilder/helix_v1_v2/tag_manager/site_manager/static/www.eczee.fr/404.html</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -502,7 +502,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>/Users/sbws_user/Documents/Webbuilder/20April/TagManger/helix_v1_v2/tag_manager/site_manager/static/site_manager/samples/www.eczee.fr/vivre-ma-dermatite-atopique/index.html</t>
+          <t>/Users/sbws_user/Documents/Custom_to_Webbuilder/helix_v1_v2/tag_manager/site_manager/static/www.eczee.fr/vivre-ma-dermatite-atopique/index.html</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -531,7 +531,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>/Users/sbws_user/Documents/Webbuilder/20April/TagManger/helix_v1_v2/tag_manager/site_manager/static/site_manager/samples/www.eczee.fr/conditions-generales-dutilisation/index.html</t>
+          <t>/Users/sbws_user/Documents/Custom_to_Webbuilder/helix_v1_v2/tag_manager/site_manager/static/www.eczee.fr/conditions-generales-dutilisation/index.html</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -560,7 +560,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>/Users/sbws_user/Documents/Webbuilder/20April/TagManger/helix_v1_v2/tag_manager/site_manager/static/site_manager/samples/www.eczee.fr/safari-pinned-tab/index.html</t>
+          <t>/Users/sbws_user/Documents/Custom_to_Webbuilder/helix_v1_v2/tag_manager/site_manager/static/www.eczee.fr/safari-pinned-tab/index.html</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -589,7 +589,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>/Users/sbws_user/Documents/Webbuilder/20April/TagManger/helix_v1_v2/tag_manager/site_manager/static/site_manager/samples/www.eczee.fr/frontpage/index.html</t>
+          <t>/Users/sbws_user/Documents/Custom_to_Webbuilder/helix_v1_v2/tag_manager/site_manager/static/www.eczee.fr/frontpage/index.html</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -617,12 +617,16 @@
           <t>PP-UNP-FRA-0506</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>keywords1, keywords2, keywords3, seo</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>/Users/sbws_user/Documents/Webbuilder/20April/TagManger/helix_v1_v2/tag_manager/site_manager/static/site_manager/samples/www.eczee.fr/traiter-ma-dermatite-atopique/index.html</t>
+          <t>/Users/sbws_user/Documents/Custom_to_Webbuilder/helix_v1_v2/tag_manager/site_manager/static/www.eczee.fr/traiter-ma-dermatite-atopique/index.html</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -642,12 +646,16 @@
           <t>PP-UNP-FRA-0506</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>dummy, dummyseo, keywords1, keywords2, keywords3</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>/Users/sbws_user/Documents/Webbuilder/20April/TagManger/helix_v1_v2/tag_manager/site_manager/static/site_manager/samples/www.eczee.fr/errors/404.html</t>
+          <t>/Users/sbws_user/Documents/Custom_to_Webbuilder/helix_v1_v2/tag_manager/site_manager/static/www.eczee.fr/errors/404.html</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -676,7 +684,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>/Users/sbws_user/Documents/Webbuilder/20April/TagManger/helix_v1_v2/tag_manager/site_manager/static/site_manager/samples/www.eczee.fr/comprendre-la-dermatite-atopique/index.html</t>
+          <t>/Users/sbws_user/Documents/Custom_to_Webbuilder/helix_v1_v2/tag_manager/site_manager/static/www.eczee.fr/comprendre-la-dermatite-atopique/index.html</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -701,7 +709,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>/Users/sbws_user/Documents/Webbuilder/20April/TagManger/helix_v1_v2/tag_manager/site_manager/static/site_manager/samples/www.eczee.fr/cdn-cgi/l/email-protection/index.html</t>
+          <t>/Users/sbws_user/Documents/Custom_to_Webbuilder/helix_v1_v2/tag_manager/site_manager/static/www.eczee.fr/cdn-cgi/l/email-protection/index.html</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -722,7 +730,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>/Users/sbws_user/Documents/Webbuilder/20April/TagManger/helix_v1_v2/tag_manager/site_manager/static/site_manager/samples/www.eczee.fr/404/index.html</t>
+          <t>/Users/sbws_user/Documents/Custom_to_Webbuilder/helix_v1_v2/tag_manager/site_manager/static/www.eczee.fr/404/index.html</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">

</xml_diff>